<commit_message>
Implement user creation functionality in Excel file
</commit_message>
<xml_diff>
--- a/Dados-login.xlsx
+++ b/Dados-login.xlsx
@@ -15,7 +15,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="25">
+  <si>
+    <t>Id</t>
+  </si>
   <si>
     <t>Nome</t>
   </si>
@@ -78,6 +81,15 @@
   </si>
   <si>
     <t>123@dxd</t>
+  </si>
+  <si>
+    <t>Lokan</t>
+  </si>
+  <si>
+    <t>lk@gmail.com</t>
+  </si>
+  <si>
+    <t>123@2d</t>
   </si>
 </sst>
 </file>
@@ -417,15 +429,16 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="14.28515625" customWidth="true" style="0"/>
     <col min="2" max="2" width="24.85546875" customWidth="true" style="0"/>
-    <col min="3" max="3" width="15.7109375" customWidth="true" style="0"/>
+    <col min="3" max="3" width="28.85546875" customWidth="true" style="0"/>
+    <col min="4" max="4" width="16.140625" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -435,10 +448,13 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="D1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -446,10 +462,13 @@
       <c r="C2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
+      <c r="D2" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3">
+        <v>2</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -457,10 +476,13 @@
       <c r="C3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
+      <c r="D3" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4">
+        <v>3</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
@@ -468,10 +490,13 @@
       <c r="C4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
+      <c r="D4" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5">
+        <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>13</v>
@@ -479,10 +504,13 @@
       <c r="C5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
+      <c r="D5" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6">
+        <v>5</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
@@ -490,16 +518,36 @@
       <c r="C6" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
+      <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
         <v>19</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C7" t="s">
         <v>20</v>
+      </c>
+      <c r="D7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>